<commit_message>
Add custom colors, update inference script, and clean up tracked files
</commit_message>
<xml_diff>
--- a/Cheque_details.xlsx
+++ b/Cheque_details.xlsx
@@ -37,22 +37,22 @@
     <t>Signature</t>
   </si>
   <si>
-    <t>E@6%</t>
-  </si>
-  <si>
-    <t>300020101088412</t>
-  </si>
-  <si>
-    <t>SYNB0003011</t>
-  </si>
-  <si>
-    <t>₹ 2500,0000/-</t>
-  </si>
-  <si>
-    <t>U083660U 5000250332 290062U 31</t>
-  </si>
-  <si>
-    <t>02/24/95</t>
+    <t>AXIS BANK LTD</t>
+  </si>
+  <si>
+    <t>911010049001545</t>
+  </si>
+  <si>
+    <t>UTIB0000426</t>
+  </si>
+  <si>
+    <t>₹ 30,000/-</t>
+  </si>
+  <si>
+    <t>U309141U 5002110128 426160U 31</t>
+  </si>
+  <si>
+    <t>25/01/2016</t>
   </si>
   <si>
     <t>True</t>

</xml_diff>